<commit_message>
test: the parts sets files, frozen-held and struct-held taken again on both Excels over files whose frozen panes have no cursor: the same answers, and both save the cursor on A1 so
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/parts/files/after-copy.xlsx
+++ b/test/excel/parts/files/after-copy.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Library/Containers/com.microsoft.Excel/Data/tmp/fparts-93983/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mike/Library/Containers/com.microsoft.Excel/Data/tmp/fsave-27467/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4CA30382-4EFA-1148-BA97-BAC2A51920D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4392278F-7EE3-B545-9C4C-E4FE0AE1422C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>